<commit_message>
Nueva version complementaria version uno, piloto sin pruebas
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diot en 0 ext\Desktop\Diot en 0 ext online\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diot en 0 ext\Desktop\Diot en 0 ext online complementaria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02B4FA50-52B0-4FD0-9F5E-BB5136BA5643}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D91E657-3D7D-4E16-9D2B-9ECEE0CCC592}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="26">
   <si>
     <t>RFC</t>
   </si>
@@ -90,6 +90,15 @@
   </si>
   <si>
     <t>COMPLEMENTARIA</t>
+  </si>
+  <si>
+    <t>Si</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>??</t>
   </si>
 </sst>
 </file>
@@ -125,43 +134,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -448,16 +429,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="42.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="41.88671875" customWidth="1"/>
     <col min="5" max="5" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -479,8 +461,11 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -499,8 +484,11 @@
       <c r="G2">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -519,8 +507,11 @@
       <c r="G3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -539,8 +530,11 @@
       <c r="G4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -559,83 +553,33 @@
       <c r="G5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6">
-        <v>2024</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7">
-        <v>2024</v>
-      </c>
-      <c r="G7">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8">
-        <v>2024</v>
-      </c>
-      <c r="G8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9">
-        <v>2024</v>
-      </c>
-      <c r="G9">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" t="s">
         <v>17</v>
       </c>
     </row>
@@ -647,168 +591,293 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="51.109375" customWidth="1"/>
-    <col min="4" max="4" width="20.109375" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="1"/>
+    <col min="4" max="4" width="20.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="11.5546875" style="2"/>
+    <col min="8" max="8" width="18.77734375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="2">
         <v>2025</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="2">
         <v>2</v>
       </c>
+      <c r="H2" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="2">
         <v>2025</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="2">
         <v>2</v>
       </c>
+      <c r="H3" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="2">
+        <v>2025</v>
+      </c>
+      <c r="G4" s="2">
+        <v>2</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="2">
+        <v>2025</v>
+      </c>
+      <c r="G5" s="2">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="2">
         <v>2024</v>
       </c>
-      <c r="G4">
+      <c r="G6" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="H6" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5">
+      <c r="F7" s="2">
         <v>2024</v>
       </c>
-      <c r="G5">
+      <c r="G7" s="2">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="H7" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F6">
+      <c r="F8" s="2">
         <v>2024</v>
       </c>
-      <c r="G6">
+      <c r="G8" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="H8" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F7">
+      <c r="F9" s="2">
         <v>2024</v>
       </c>
-      <c r="G7">
+      <c r="G9" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
+      <c r="H9" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21"/>
+      <c r="B21"/>
+      <c r="C21"/>
+      <c r="D21"/>
+      <c r="E21"/>
+      <c r="F21"/>
+      <c r="G21"/>
+      <c r="H21"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22"/>
+      <c r="B22"/>
+      <c r="C22"/>
+      <c r="D22"/>
+      <c r="E22"/>
+      <c r="F22"/>
+      <c r="G22"/>
+      <c r="H22"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23"/>
+      <c r="B23"/>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
+      <c r="F23"/>
+      <c r="G23"/>
+      <c r="H23"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24"/>
+      <c r="B24"/>
+      <c r="C24"/>
+      <c r="D24"/>
+      <c r="E24"/>
+      <c r="F24"/>
+      <c r="G24"/>
+      <c r="H24"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25"/>
+      <c r="B25"/>
+      <c r="C25"/>
+      <c r="D25"/>
+      <c r="E25"/>
+      <c r="F25"/>
+      <c r="G25"/>
+      <c r="H25"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26"/>
+      <c r="B26"/>
+      <c r="C26"/>
+      <c r="D26"/>
+      <c r="E26"/>
+      <c r="F26"/>
+      <c r="G26"/>
+      <c r="H26"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A6">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A3 A5">
-    <cfRule type="duplicateValues" dxfId="1" priority="20"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A4">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="A1:A3">
+    <cfRule type="duplicateValues" dxfId="0" priority="23"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>